<commit_message>
Renamed problem statement and add addtional reqs
</commit_message>
<xml_diff>
--- a/Requirements.xlsx
+++ b/Requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nps01-my.sharepoint.com/personal/luke_smith_nps_edu/Documents/Documents/GitHub/SE4003-Capstone-U2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_F25DC773A252ABDACC104892715C7D4C5BDE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FDC10CB-F154-46C0-B256-ECBE2153DD67}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_F25DC773A252ABDACC104892715C7D4C5BDE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CD154A4-A96D-4468-A9B5-CC013B2E0DFC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1725" yWindow="2685" windowWidth="13080" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Name</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Simulation</t>
   </si>
   <si>
-    <t>iRobot Platfrom</t>
-  </si>
-  <si>
     <t>Code shall be written in python</t>
   </si>
   <si>
@@ -66,19 +63,76 @@
     <t>The system shall operate simulation environment</t>
   </si>
   <si>
-    <t>The system proof of concept shall be a iRobot compatable Roomba</t>
-  </si>
-  <si>
     <t>ROS Topics</t>
   </si>
   <si>
     <t>ROS Nodes</t>
   </si>
   <si>
-    <t>The system shall subscribe and publishs to relevelent ROS topics</t>
-  </si>
-  <si>
     <t>The system shall consist of ROS nodes</t>
+  </si>
+  <si>
+    <t>The system shall subscribe and publish to relevant ROS topics</t>
+  </si>
+  <si>
+    <t>iRobot Platform</t>
+  </si>
+  <si>
+    <t>The system proof of concept shall be a iRobot compatible Roomba</t>
+  </si>
+  <si>
+    <t>ROS Topics Documentation</t>
+  </si>
+  <si>
+    <t>ROS Position</t>
+  </si>
+  <si>
+    <t>ROS Map</t>
+  </si>
+  <si>
+    <t>ROS Services</t>
+  </si>
+  <si>
+    <t>Wall</t>
+  </si>
+  <si>
+    <t>Communication</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>The system shall communicate with operator</t>
+  </si>
+  <si>
+    <t>The system shall report completion or termination of task</t>
+  </si>
+  <si>
+    <t>ROS Log</t>
+  </si>
+  <si>
+    <t>The system shall log a time series topics files</t>
+  </si>
+  <si>
+    <t>The system shall determine position relative to start while exploring</t>
+  </si>
+  <si>
+    <t>The system shall determine topography of room</t>
+  </si>
+  <si>
+    <t>Stuck</t>
+  </si>
+  <si>
+    <t>The system shall determine when movement is attempted but not change of position occurs</t>
+  </si>
+  <si>
+    <t>The system internal interfaces shall be documented topics or services when passing information between nodes</t>
+  </si>
+  <si>
+    <t>The system shall detect vertical obstacles of at least {} cm</t>
+  </si>
+  <si>
+    <t>Terrain</t>
   </si>
 </sst>
 </file>
@@ -396,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
@@ -421,7 +475,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -429,7 +483,7 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -442,31 +496,105 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>